<commit_message>
ready for pipetting 1000reactions 03.20
</commit_message>
<xml_diff>
--- a/zeus-pipetter/NPs/2023_03_15-reaction_template_for_robot_Yankai.xlsx
+++ b/zeus-pipetter/NPs/2023_03_15-reaction_template_for_robot_Yankai.xlsx
@@ -19101,7 +19101,7 @@
         <v>4.5</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>2017</v>
+        <v>2021</v>
       </c>
       <c r="H2" s="7" t="inlineStr">
         <is>
@@ -19109,7 +19109,7 @@
         </is>
       </c>
       <c r="I2" s="7" t="n">
-        <v>8069.1</v>
+        <v>7864.8</v>
       </c>
     </row>
     <row r="3">
@@ -19140,7 +19140,7 @@
         <v>4.5</v>
       </c>
       <c r="G3" s="7" t="n">
-        <v>2097</v>
+        <v>2099</v>
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
@@ -19148,7 +19148,7 @@
         </is>
       </c>
       <c r="I3" s="7" t="n">
-        <v>3983.5</v>
+        <v>3881.3</v>
       </c>
     </row>
     <row r="4">
@@ -19179,7 +19179,7 @@
         <v>4.5</v>
       </c>
       <c r="G4" s="7" t="n">
-        <v>1908</v>
+        <v>1914</v>
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
@@ -19187,7 +19187,7 @@
         </is>
       </c>
       <c r="I4" s="7" t="n">
-        <v>13635.7</v>
+        <v>13329.3</v>
       </c>
     </row>
     <row r="5">
@@ -19218,7 +19218,7 @@
         <v>4.5</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>2087</v>
+        <v>2091</v>
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
@@ -19226,7 +19226,7 @@
         </is>
       </c>
       <c r="I5" s="7" t="n">
-        <v>4494.2</v>
+        <v>4289.9</v>
       </c>
     </row>
     <row r="6">
@@ -19257,7 +19257,7 @@
         <v>9</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>2045</v>
+        <v>2049</v>
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
@@ -19265,7 +19265,7 @@
         </is>
       </c>
       <c r="I6" s="7" t="n">
-        <v>6639.1</v>
+        <v>6434.8</v>
       </c>
     </row>
     <row r="7">
@@ -19296,7 +19296,7 @@
         <v>20</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>1970</v>
+        <v>1975</v>
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
@@ -19304,7 +19304,7 @@
         </is>
       </c>
       <c r="I7" s="7" t="n">
-        <v>10469.4</v>
+        <v>10214</v>
       </c>
     </row>
   </sheetData>

</xml_diff>